<commit_message>
Timothy/Cleaned up and documented the main method
</commit_message>
<xml_diff>
--- a/output data/eclat_validation.xlsx
+++ b/output data/eclat_validation.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>114420</v>
+        <v>114395</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14980</v>
+        <v>14879</v>
       </c>
     </row>
     <row r="4">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1225</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="7">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6716288384512683</v>
+        <v>0.6714396128772095</v>
       </c>
     </row>
   </sheetData>
@@ -542,7 +542,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>event_rank=High</t>
+          <t>venue=T-Mobile Park, event_rank=High</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -552,7 +552,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, event_rank=High</t>
+          <t>event_rank=High</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11823</v>
+        <v>11648</v>
       </c>
     </row>
     <row r="7">
@@ -586,37 +586,37 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8344</v>
+        <v>8898</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>position=Cashier</t>
+          <t>position=Stock Associate</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8124</v>
+        <v>8545</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, event_rank=High, availability=Full-time</t>
+          <t>schedule=Mon-Wed 8AM-2PM</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8060</v>
+        <v>7965</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>event_rank=High, availability=Full-time</t>
+          <t>venue=T-Mobile Park, event_rank=High, availability=Full-time</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8060</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="11">
@@ -626,27 +626,27 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8060</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>position=Assistant Manager</t>
+          <t>event_rank=High, availability=Full-time</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8029</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>position=Stock Associate</t>
+          <t>position=Assistant Manager</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7993</v>
+        <v>7705</v>
       </c>
     </row>
     <row r="14">
@@ -656,27 +656,27 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7958</v>
+        <v>7667</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>schedule=Flexible / On-call</t>
+          <t>position=Cashier</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7926</v>
+        <v>7633</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>schedule=Mon-Fri 9AM-5PM</t>
+          <t>schedule=Flexible / On-call</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7749</v>
+        <v>7608</v>
       </c>
     </row>
   </sheetData>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11440</v>
+        <v>11340</v>
       </c>
     </row>
     <row r="3">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3540</v>
+        <v>3539</v>
       </c>
     </row>
   </sheetData>
@@ -768,47 +768,47 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2011</v>
+        <v>2221</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Stock Associate</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2011</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cashier</t>
+          <t>Assistant Manager</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1981</v>
+        <v>2010</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Assistant Manager</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1971</v>
+        <v>1821</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Stock Associate</t>
+          <t>Cashier</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1950</v>
+        <v>1696</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Timothy/Added documentation  and test code
</commit_message>
<xml_diff>
--- a/output data/eclat_validation.xlsx
+++ b/output data/eclat_validation.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>114395</v>
+        <v>115315</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14879</v>
+        <v>15012</v>
       </c>
     </row>
     <row r="4">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1227</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="7">
@@ -500,7 +500,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.6714396128772095</v>
+        <v>0.6732653876898481</v>
       </c>
     </row>
   </sheetData>
@@ -576,107 +576,107 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11648</v>
+        <v>11391</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>position=Customer Service Rep</t>
+          <t>schedule=Mon-Wed 8AM-2PM</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8898</v>
+        <v>8665</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>position=Stock Associate</t>
+          <t>position=Customer Service Rep</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8545</v>
+        <v>8506</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>schedule=Mon-Wed 8AM-2PM</t>
+          <t>position=Assistant Manager</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7965</v>
+        <v>8358</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, event_rank=High, availability=Full-time</t>
+          <t>position=Cashier</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7920</v>
+        <v>8116</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, availability=Full-time</t>
+          <t>venue=T-Mobile Park, event_rank=High, availability=Full-time</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7920</v>
+        <v>7800</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>event_rank=High, availability=Full-time</t>
+          <t>venue=T-Mobile Park, availability=Full-time</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7920</v>
+        <v>7800</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>position=Assistant Manager</t>
+          <t>event_rank=High, availability=Full-time</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7705</v>
+        <v>7800</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>position=Sales Associate</t>
+          <t>position=Stock Associate</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7667</v>
+        <v>7761</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>position=Cashier</t>
+          <t>schedule=Flexible / On-call</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7633</v>
+        <v>7709</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>schedule=Flexible / On-call</t>
+          <t>position=Sales Associate</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7608</v>
+        <v>7707</v>
       </c>
     </row>
   </sheetData>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11340</v>
+        <v>11460</v>
       </c>
     </row>
     <row r="3">
@@ -722,7 +722,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3539</v>
+        <v>3552</v>
       </c>
     </row>
   </sheetData>
@@ -764,31 +764,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Customer Service Rep</t>
+          <t>Assistant Manager</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2221</v>
+        <v>2173</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Stock Associate</t>
+          <t>Customer Service Rep</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2075</v>
+        <v>2037</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Assistant Manager</t>
+          <t>Stock Associate</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2010</v>
+        <v>1925</v>
       </c>
     </row>
     <row r="6">
@@ -798,7 +798,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1821</v>
+        <v>1918</v>
       </c>
     </row>
     <row r="7">
@@ -808,7 +808,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1696</v>
+        <v>1903</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Timothy/Trying to Validate eclat
</commit_message>
<xml_diff>
--- a/output data/eclat_validation.xlsx
+++ b/output data/eclat_validation.xlsx
@@ -450,7 +450,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>115315</v>
+        <v>928</v>
       </c>
     </row>
     <row r="3">
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -528,36 +528,50 @@
           <t>support</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>pattern_length</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park</t>
+          <t>event_rank=High</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>31140</v>
       </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, event_rank=High</t>
+          <t>event_rank=High, venue=T-Mobile Park</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>31140</v>
       </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>event_rank=High</t>
+          <t>venue=T-Mobile Park</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>31140</v>
       </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -568,6 +582,9 @@
       <c r="B5" t="n">
         <v>14364</v>
       </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -578,6 +595,9 @@
       <c r="B6" t="n">
         <v>11391</v>
       </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -588,6 +608,9 @@
       <c r="B7" t="n">
         <v>8665</v>
       </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -598,6 +621,9 @@
       <c r="B8" t="n">
         <v>8506</v>
       </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -608,6 +634,9 @@
       <c r="B9" t="n">
         <v>8358</v>
       </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -618,65 +647,86 @@
       <c r="B10" t="n">
         <v>8116</v>
       </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, event_rank=High, availability=Full-time</t>
+          <t>venue=T-Mobile Park, availability=Full-time</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>7800</v>
       </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>venue=T-Mobile Park, availability=Full-time</t>
+          <t>event_rank=High, availability=Full-time</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>7800</v>
       </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>event_rank=High, availability=Full-time</t>
+          <t>position=Stock Associate</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7800</v>
+        <v>7761</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>position=Stock Associate</t>
+          <t>schedule=Flexible / On-call</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7761</v>
+        <v>7709</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>schedule=Flexible / On-call</t>
+          <t>position=Sales Associate</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7709</v>
+        <v>7707</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>position=Sales Associate</t>
+          <t>schedule=Thu-Sun 12PM-8PM</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7707</v>
+        <v>7637</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>